<commit_message>
feat(demo): generate the showcase workbook and give it a chart (#130)
Co-authored-by: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/demo/public/showcase.xlsx
+++ b/apps/demo/public/showcase.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="948" uniqueCount="54">
   <si>
     <t xml:space="preserve">Q3 Sales Dashboard</t>
   </si>
@@ -64,13 +64,34 @@
     <t xml:space="preserve">Result</t>
   </si>
   <si>
+    <t xml:space="preserve">Values</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Key</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value</t>
+  </si>
+  <si>
     <t xml:space="preserve">SUM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alpha</t>
   </si>
   <si>
     <t xml:space="preserve">AVERAGE</t>
   </si>
   <si>
+    <t xml:space="preserve">Beta</t>
+  </si>
+  <si>
     <t xml:space="preserve">MIN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gamma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Northeast</t>
   </si>
   <si>
     <t xml:space="preserve">MAX</t>
@@ -98,27 +119,6 @@
   </si>
   <si>
     <t xml:space="preserve">End of month</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Values</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Key</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alpha</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Beta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gamma</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Northeast</t>
   </si>
   <si>
     <t xml:space="preserve">Date</t>
@@ -276,6 +276,182 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="1"/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1400" b="1"/>
+              <a:t>Revenue by region</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Dashboard!$C$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Revenue</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="4472C4"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Dashboard!$A$5:$A$8</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>North</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>South</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>East</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>West</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Dashboard!$C$5:$C$8</c:f>
+              <c:numCache>
+                <c:formatCode>"$"#,##0.00</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>386400</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>274850</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>512300</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>331200</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="150"/>
+        <c:axId val="553771648"/>
+        <c:axId val="553773184"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="553771648"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="553773184"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="553773184"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="&quot;$&quot;#,##0" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="553771648"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Revenue by region"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F11"/>
@@ -424,11 +600,12 @@
       <c r="F11" s="10"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A11:F11"/>
   </mergeCells>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -456,13 +633,13 @@
         <v>16</v>
       </c>
       <c r="E2" t="s" s="3">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="H2" t="s" s="3">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="I2" t="s" s="3">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="K2" t="s" s="3">
         <v>2</v>
@@ -470,7 +647,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s" s="11">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B3">
         <f>SUM(E3:E7)</f>
@@ -479,7 +656,7 @@
         <v>12</v>
       </c>
       <c r="H3" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="I3">
         <v>100</v>
@@ -490,7 +667,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s" s="11">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B4">
         <f>AVERAGE(E3:E7)</f>
@@ -499,7 +676,7 @@
         <v>47</v>
       </c>
       <c r="H4" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="I4">
         <v>200</v>
@@ -510,7 +687,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s" s="11">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B5">
         <f>MIN(E3:E7)</f>
@@ -519,18 +696,18 @@
         <v>8</v>
       </c>
       <c r="H5" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="I5">
         <v>300</v>
       </c>
       <c r="K5" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="11">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B6">
         <f>MAX(E3:E7)</f>
@@ -544,7 +721,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s" s="11">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="B7">
         <f>IF(B3&gt;100,"Over budget","Within budget")</f>
@@ -555,7 +732,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s" s="11">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="B8">
         <f>IFS(B4&gt;=40,"High",B4&gt;=20,"Medium",TRUE,"Low")</f>
@@ -563,7 +740,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s" s="11">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="B9">
         <f>VLOOKUP("Gamma",H3:I5,2,FALSE)</f>
@@ -571,7 +748,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s" s="11">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="B10">
         <f>COUNTIF(K3:K6,"North*")</f>
@@ -579,7 +756,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s" s="11">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="B11" s="6">
         <f>B4/B6</f>
@@ -587,7 +764,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s" s="11">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="B12">
         <f>TEXT(B4,"#,##0.00")</f>
@@ -595,7 +772,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s" s="11">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="B13" s="5">
         <f>TODAY()</f>
@@ -603,7 +780,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s" s="11">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="B14" s="5">
         <f>EOMONTH(TODAY(),0)</f>

</xml_diff>